<commit_message>
Free Lite tracker: accurate upsell (no 'points ladder', KEEP/REVIEW not KEEP/CANCEL, real card capacity), 1c example values per its own how-to, Jan/Feb months like the Command Center, .com, Amex Gold note fixed; templates.html no longer claims the free file tracks 5/24
</commit_message>
<xml_diff>
--- a/downloads/TF-Free-Lite-Card-Tracker.xlsx
+++ b/downloads/TF-Free-Lite-Card-Tracker.xlsx
@@ -11,7 +11,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card Tracker" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full version" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'How to use'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Card Tracker'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Card Tracker'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Full version'!$A$1:$C$11</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,8 +98,76 @@
       <sz val="12"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00D5DBE7"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C8A24A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B2333"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00616B7D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B2333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B2545"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00616B7D"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00616B7D"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F1E3D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000E7C7B"/>
+      <sz val="12"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -116,8 +189,18 @@
         <fgColor rgb="000B2A4A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F1E3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0016294F"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -139,11 +222,25 @@
         <color rgb="00D9D4C7"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="0016294F"/>
+      </left>
+      <right style="thin">
+        <color rgb="0016294F"/>
+      </right>
+      <top style="thin">
+        <color rgb="0016294F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C8A24A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -188,6 +285,53 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -550,8 +694,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C8A24A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -561,55 +706,55 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Free Credit Card Tracker</t>
         </is>
       </c>
-      <c r="B1" s="15" t="n"/>
-      <c r="C1" s="15" t="n"/>
+      <c r="B1" s="22" t="n"/>
+      <c r="C1" s="22" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Start here: 1 minute.</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n"/>
-      <c r="C2" s="15" t="n"/>
+      <c r="B2" s="23" t="n"/>
+      <c r="C2" s="23" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Travel &amp; Finance  ·  travelfinancetips</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="n"/>
-      <c r="C3" s="15" t="n"/>
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Travel &amp; Finance  ·  travelfinancetips.com</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n"/>
+      <c r="C3" s="24" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>1.  Open the 'Card Tracker' tab and replace the example rows with your cards (up to 5).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>2.  Pick the month your annual fee posts from the dropdown.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>3.  Estimate your points value: points × cents per point ÷ 100 (1¢ is a safe floor).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>4.  Check it a month before each fee posts. If the value you use is below the fee, ask about a downgrade.</t>
         </is>
@@ -619,29 +764,40 @@
       <c r="B9" s="18" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>Want the math done for you? See the 'Full version' tab.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>Educational only, not financial advice. Card terms and fees are set by the issuer and change.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;"Arial"&amp;8 Travel &amp; Finance Tips  ·  travelfinancetips.com&amp;R&amp;"Arial"&amp;8 &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0016294F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -652,128 +808,128 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="26" t="inlineStr">
         <is>
           <t>TRAVEL &amp; FINANCE TIPS  —  Free Credit Card Lite Tracker</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>Track up to 5 cards: fees, when the annual fee hits, and your points. Keep it simple.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>Card Name</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>Annual Fee</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>Fee Month</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="28" t="inlineStr">
         <is>
           <t>Points/Miles</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="28" t="inlineStr">
         <is>
           <t>Est. Point Value ($)</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="28" t="inlineStr">
         <is>
           <t>Notes / Bonus Deadline</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Chase Sapphire Preferred</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="30" t="n">
         <v>95</v>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>October</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n">
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="n">
         <v>62000</v>
       </c>
-      <c r="F6" s="5" t="n">
-        <v>930</v>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="F6" s="30" t="n">
+        <v>620</v>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
         <is>
           <t>Keep — $50 hotel + points cover fee</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Amex Gold</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="30" t="n">
         <v>325</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n">
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="n">
         <v>48000</v>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>720</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Dining + grocery credits offset fee</t>
+      <c r="F7" s="30" t="n">
+        <v>480</v>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>Dining + Uber Cash credits offset fee</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Capital One VentureX</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Capital One Venture X</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="n">
         <v>395</v>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>January</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n">
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="n">
         <v>90000</v>
       </c>
-      <c r="F8" s="5" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="F8" s="30" t="n">
+        <v>900</v>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
         <is>
           <t>$300 travel credit + anniversary miles</t>
         </is>
@@ -796,34 +952,34 @@
       <c r="G10" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="34">
         <f>SUM(C6:C10)</f>
         <v/>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>Total point value:</t>
         </is>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="34">
         <f>SUM(F6:F10)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Want the full system? The Credit Card Wealth Bundle adds 5/24 tracking, auto KEEP/CANCEL verdicts, a rewards optimizer &amp; points ladder →  travelfinancetips.com/templates</t>
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>Want the full system? The Credit Card Wealth Bundle adds 5/24 tracking, keep-or-review verdicts, a rewards optimizer and a points tracker with expiry alerts →  travelfinancetips.com/templates</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>Educational tool, not financial advice. © Travel &amp; Finance Tips</t>
         </is>
@@ -838,7 +994,7 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D6:D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"January,February,March,April,May,June,July,August,September,October,November,December"</formula1>
+      <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
     <dataValidation sqref="C6:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Numbers only" error="Enter a dollar amount (0 or more), no $ sign needed." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
@@ -847,113 +1003,124 @@
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;"Arial"&amp;8 Travel &amp; Finance Tips  ·  travelfinancetips.com&amp;R&amp;"Arial"&amp;8 &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C8A24A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>What the full version adds</t>
         </is>
       </c>
-      <c r="B1" s="15" t="n"/>
-      <c r="C1" s="15" t="n"/>
+      <c r="B1" s="22" t="n"/>
+      <c r="C1" s="22" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>The Credit Card Wealth Bundle: 4 templates, $29.</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n"/>
-      <c r="C2" s="15" t="n"/>
+      <c r="B2" s="23" t="n"/>
+      <c r="C2" s="23" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Travel &amp; Finance  ·  travelfinancetips</t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="n"/>
-      <c r="C3" s="15" t="n"/>
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Travel &amp; Finance  ·  travelfinancetips.com</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n"/>
+      <c r="C3" s="24" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
         <is>
           <t>Annual-Fee ROI Calculator</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>Keep / borderline / reconsider verdict for every card, with a one-glance scorecard.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>Credit Card Command Center</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>Every card, fee month, unused credits, points value and your 5/24 count in one place.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>Points &amp; Miles Tracker</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>All balances, expiry warnings, and a redemption log that grades each redemption.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>Rewards Optimizer</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>Tells you which card to use for each spend category and what it's worth per year.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>Unlimited cards</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>The free tracker holds 5. The full versions hold 12-30.</t>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>Room to grow</t>
+        </is>
+      </c>
+      <c r="C9" s="42" t="inlineStr">
+        <is>
+          <t>The free tracker holds 5 cards. The Command Center holds 25, the ROI Calculator 12, and the Points Tracker 30 programs.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="40" t="inlineStr">
         <is>
           <t>Get it: travelfinancetips.com/templates.html</t>
         </is>
@@ -963,6 +1130,16 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId1"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;"Arial"&amp;8 Travel &amp; Finance Tips  ·  travelfinancetips.com&amp;R&amp;"Arial"&amp;8 &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>